<commit_message>
Finish Figure 2 and attribute both figures at point of use
Rename the Figure 2 legend to the ASPE entry-cost scenarios, add a
dashed medium break-even marker at $15.8M, and add the exported image.
Add point-of-use attribution for Figures 1 and 2 and log row 21.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/required-uplift-u.xlsx
+++ b/analysis/required-uplift-u.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allenmehr/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allenmehr/Documents/GitHub/allen-mehr/analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69FF2B3-58C8-3F44-85DC-6040F96569DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{796D2F9F-C186-FC42-91E7-BD92F2414DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>Required uplift u by scenario</t>
   </si>
@@ -81,6 +81,12 @@
   </si>
   <si>
     <t>Revenue runs from $1M through $25M in $1M steps</t>
+  </si>
+  <si>
+    <t>Medium break-even marker (vertical line on chart)</t>
+  </si>
+  <si>
+    <t>u</t>
   </si>
 </sst>
 </file>
@@ -231,10 +237,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -391,13 +397,13 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="smoothMarker"/>
+        <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Low</c:v>
+            <c:v>Low entry cost (ASPE)</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
@@ -580,7 +586,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-F120-0D4E-8F09-FA18DAC6E71F}"/>
@@ -591,7 +597,7 @@
           <c:idx val="2"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Medium</c:v>
+            <c:v>Medium entry cost (ASPE)</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
@@ -774,7 +780,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-F120-0D4E-8F09-FA18DAC6E71F}"/>
@@ -785,7 +791,7 @@
           <c:idx val="3"/>
           <c:order val="2"/>
           <c:tx>
-            <c:v>High</c:v>
+            <c:v>High entry cost (ASPE)</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
@@ -968,10 +974,66 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-F120-0D4E-8F09-FA18DAC6E71F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>Medium break-even ($15.8M)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="5B6573"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Required Uplift'!$F$14:$F$15</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>15800141.379310345</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15800141.379310345</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Required Uplift'!$G$14:$G$15</c:f>
+              <c:numCache>
+                <c:formatCode>0.0000;\-0.0000;0</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2C47-2648-814B-38386BF6C29A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1868,10 +1930,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>330200</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1897,10 +1959,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2082,7 +2140,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
@@ -2090,22 +2148,22 @@
     <col min="6" max="14" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
@@ -2113,7 +2171,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>4</v>
       </c>
@@ -2124,7 +2182,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -2136,7 +2194,7 @@
         <v>10209489.655172415</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>8</v>
       </c>
@@ -2148,7 +2206,7 @@
         <v>15800141.379310345</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>9</v>
       </c>
@@ -2160,12 +2218,15 @@
         <v>21066856.896551725</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
         <v>11</v>
       </c>
@@ -2178,8 +2239,14 @@
       <c r="D13" s="12" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F13" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="11">
         <v>1000000</v>
       </c>
@@ -2195,8 +2262,15 @@
         <f>MAX(0,$B$10/A14-0.58)</f>
         <v>11.638776999999999</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F14" s="11">
+        <f>$C$9</f>
+        <v>15800141.379310345</v>
+      </c>
+      <c r="G14" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="11">
         <v>2000000</v>
       </c>
@@ -2212,8 +2286,15 @@
         <f t="shared" ref="D15:D38" si="2">MAX(0,$B$10/A15-0.58)</f>
         <v>5.5293884999999996</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F15" s="11">
+        <f>$C$9</f>
+        <v>15800141.379310345</v>
+      </c>
+      <c r="G15" s="10">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="11">
         <v>3000000</v>
       </c>

</xml_diff>